<commit_message>
feat(dialogue): drive NPC dialogue from table with camera switch
NPC with a dialogueId opens DialogueUI in table mode and blends to an
optional dialogue camera, restoring the previous camera on close.
Adds Dialogue table data and text box sprite import.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Table/Excel/Dialogue.xlsx
+++ b/Table/Excel/Dialogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TokTak\Desktop\Local\Unity\LOTW\LOTW\Table\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{21C6A091-4D48-494A-89B4-C821145B2CA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{608D3147-EF93-4159-AD49-DB2720E52C66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{975E7E8E-6DC6-42D4-B3B5-80E8F47AC915}"/>
   </bookViews>
@@ -16,61 +16,77 @@
     <sheet name="Dialogue" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Dialogue!$A$1:$F$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Dialogue!$B$2:$G$7</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="20">
+  <si>
+    <t>SpeakerId</t>
+  </si>
+  <si>
+    <t>SpeakerName</t>
+  </si>
+  <si>
+    <t>Text</t>
+  </si>
+  <si>
+    <t>NextId</t>
+  </si>
+  <si>
+    <t>ChoiceIds</t>
+  </si>
+  <si>
+    <t>npc_shopkeeper</t>
+  </si>
+  <si>
+    <t>상점 주인</t>
+  </si>
+  <si>
+    <t>어서오세요! 무엇을 도와드릴까요?</t>
+  </si>
+  <si>
+    <t>2,3</t>
+  </si>
+  <si>
+    <t>player</t>
+  </si>
+  <si>
+    <t>플레이어</t>
+  </si>
+  <si>
+    <t>꽃을 좀 구경해도 될까요?</t>
+  </si>
+  <si>
+    <t>아니요, 그냥 지나가는 길이에요.</t>
+  </si>
+  <si>
+    <t>물론이죠! 오늘 들어온 장미가 특히 예쁘답니다.</t>
+  </si>
+  <si>
+    <t>그렇군요. 또 들러주세요!</t>
+  </si>
+  <si>
+    <t>합계</t>
+  </si>
+  <si>
+    <t>평균</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>누계</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>개수</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
   <si>
     <t>DataId</t>
-  </si>
-  <si>
-    <t>SpeakerId</t>
-  </si>
-  <si>
-    <t>SpeakerName</t>
-  </si>
-  <si>
-    <t>Text</t>
-  </si>
-  <si>
-    <t>NextId</t>
-  </si>
-  <si>
-    <t>ChoiceIds</t>
-  </si>
-  <si>
-    <t>npc_shopkeeper</t>
-  </si>
-  <si>
-    <t>상점 주인</t>
-  </si>
-  <si>
-    <t>어서오세요! 무엇을 도와드릴까요?</t>
-  </si>
-  <si>
-    <t>2,3</t>
-  </si>
-  <si>
-    <t>player</t>
-  </si>
-  <si>
-    <t>플레이어</t>
-  </si>
-  <si>
-    <t>꽃을 좀 구경해도 될까요?</t>
-  </si>
-  <si>
-    <t>아니요, 그냥 지나가는 길이에요.</t>
-  </si>
-  <si>
-    <t>물론이죠! 오늘 들어온 장미가 특히 예쁘답니다.</t>
-  </si>
-  <si>
-    <t>그렇군요. 또 들러주세요!</t>
+    <phoneticPr fontId="18" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -661,9 +677,12 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -710,7 +729,32 @@
     <cellStyle name="출력" xfId="10" builtinId="21" customBuiltin="1"/>
     <cellStyle name="표준" xfId="0" builtinId="0" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="8">
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -721,6 +765,21 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5EA09B9D-CBAC-4460-AFA5-93C78FE52170}" name="표1" displayName="표1" ref="B2:G7" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
+  <autoFilter ref="B2:G7" xr:uid="{9D75DD4E-1EF1-4D17-8724-351AB6C1FED7}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{3DF22982-DB7A-4D9C-9F71-569FF9C62119}" name="DataId" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{B1048F0D-B7C5-4595-8ADC-9E313640957A}" name="SpeakerId" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{A665EDEC-2932-42F3-A63D-B60BF5D53D12}" name="SpeakerName" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{B2ABE83A-927C-4961-A82A-DA6CF3FE0D0E}" name="Text" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{661C07ED-3865-45B5-BEB5-98695189D34D}" name="NextId" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{B842CA46-F4C9-4028-AA4E-41A5E2C099EB}" name="ChoiceIds" dataDxfId="2"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1020,127 +1079,134 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66214232-5F92-488A-8B78-1F28277602D4}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="B2:G7"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18.125" customWidth="1"/>
     <col min="3" max="3" width="15.25" customWidth="1"/>
-    <col min="4" max="4" width="44.625" customWidth="1"/>
-    <col min="5" max="5" width="11.875" customWidth="1"/>
-    <col min="6" max="6" width="10.5" customWidth="1"/>
+    <col min="4" max="4" width="18.625" customWidth="1"/>
+    <col min="5" max="5" width="44.75" customWidth="1"/>
+    <col min="6" max="6" width="16.5" customWidth="1"/>
+    <col min="7" max="7" width="12.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="2" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+    </row>
+    <row r="3" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="D3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="1">
+        <v>-1</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="4" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="1">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="1">
+        <v>4</v>
+      </c>
+      <c r="G4" s="1"/>
+    </row>
+    <row r="5" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="1">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="1">
+        <v>5</v>
+      </c>
+      <c r="G5" s="1"/>
+    </row>
+    <row r="6" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="1">
+        <v>4</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2">
+      <c r="E6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="1">
         <v>-1</v>
       </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
+      <c r="G6" s="1"/>
     </row>
-    <row r="3" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4">
+    <row r="7" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="1">
         <v>5</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="E7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="E5">
+      <c r="F7" s="1">
         <v>-1</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" t="s">
-        <v>7</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6">
-        <v>-1</v>
-      </c>
+      <c r="G7" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F6" xr:uid="{9D75DD4E-1EF1-4D17-8724-351AB6C1FED7}"/>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(story): sequence player, prologue and time slots
- Sequence table (dialogue/wait/fade/camera/scene/actions steps linked by nextId)
- SequencePlayer survives scene loads and blocks player input while playing
- Dialogue action sequence:id, SequenceTrigger, new game plays the prologue
- SceneTransitionManager.FadeAsync for fades without scene loads
- Prologue draft (night bus, mayor briefing, 7am office) and evening transition
- TimeSlot enum, table validation tests

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Table/Excel/Dialogue.xlsx
+++ b/Table/Excel/Dialogue.xlsx
@@ -125,8 +125,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DialogueTable" displayName="DialogueTable" ref="A1:H51" headerRowCount="1">
-  <autoFilter ref="A1:H51"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DialogueTable" displayName="DialogueTable" ref="A1:H61" headerRowCount="1">
+  <autoFilter ref="A1:H61"/>
   <tableColumns count="8">
     <tableColumn id="1" name="DataId"/>
     <tableColumn id="2" name="SpeakerId"/>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1497,6 +1497,217 @@
         <v>-1</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>9000</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr"/>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>12월 16일, 일요일 밤.</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>9001</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>9001</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr"/>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>깨끗한 빨간 버스 한 대가 보라 마을에 도착했다.</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>9002</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>9002</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr"/>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>코트에 모자를 쓴 누군가가 짐을 들고 긴 언덕길을 오른다.</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>9010</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>npc_mayor</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>촌장</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>탐정 양반! 기다리고 있었네.</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>9011</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>9011</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>npc_mayor</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>촌장</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>지난 수요일, 12월 12일에 마을의 보물이 사라진 걸 알았지.</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>9012</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>9012</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>npc_mayor</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>촌장</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>무엇보다 범인을 찾는 게 먼저일세. 범인은... 분명 이 마을 주민이야.</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>9013</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>9013</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>npc_mayor</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>촌장</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>그럼 잘 부탁하네! 난 이만 바빠서.</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>meet:npc_mayor;addNote:101;startQuest:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>9020</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr"/>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>오전 7시. 1층 간판을 뒤집었다.</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>9021</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>9021</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr"/>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>'탐정 사무소 오픈. 도움이 필요하다면 언제든지 방문 환영.'</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>9022</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>9022</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr"/>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>...공기가 차갑다.</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat(world): inspectables, save action, talk counts and quest marks
- Inspectable opens a narration dialogue; desk draft rows 9100-9103
- Dialogue action save stores the current slot; HUD shows a saved toast
- NPC characterId (set for the six Plaza NPCs) and talk.{id} counter flag
- Gumman small talk varies by talk count (rows 1110-1113)
- QuestMarkIndicator shows a sweat mark for not-started quests in the
  current chapter; editor menu adds it to PF_NPC_Base
- Sweat sprites use PPU 25

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Table/Excel/Dialogue.xlsx
+++ b/Table/Excel/Dialogue.xlsx
@@ -125,8 +125,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DialogueTable" displayName="DialogueTable" ref="A1:H61" headerRowCount="1">
-  <autoFilter ref="A1:H61"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DialogueTable" displayName="DialogueTable" ref="A1:H68" headerRowCount="1">
+  <autoFilter ref="A1:H68"/>
   <tableColumns count="8">
     <tableColumn id="1" name="DataId"/>
     <tableColumn id="2" name="SpeakerId"/>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -439,7 +439,7 @@
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
     <col width="44" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -760,23 +760,18 @@
       <c r="A14" t="n">
         <v>1110</v>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>npc_gumman</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>먼저 인사라도 건네보라고!</t>
-        </is>
-      </c>
       <c r="E14" t="n">
         <v>-1</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1111,1112,1113</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>1120</v>
+        <v>1111</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -785,309 +780,309 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>아직 아는 게 없어.</t>
+          <t>먼저 인사라도 건네보라고!</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>1100</v>
+        <v>-1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>flag:talk.npc_gumman&lt;=1</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
+        <v>1112</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>npc_gumman</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>이 마을 사람들, 겉보기보다 말이 많아. 들어주기만 하면 돼.</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>flag:talk.npc_gumman==2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>1113</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>npc_gumman</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>또 왔어? 탐정 일은 발로 하는 거라고.</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>1120</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>npc_gumman</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>아직 아는 게 없어.</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
         <v>1200</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>npc_catty</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>우리 마을에 박물관 있는 거 아세요?
 진짜 짱이거든요.</t>
         </is>
       </c>
-      <c r="E16" t="n">
+      <c r="E19" t="n">
         <v>1201</v>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>meet:npc_catty</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="n">
+    <row r="20">
+      <c r="A20" t="n">
         <v>1201</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>npc_catty</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>나중에 꼭 가보세요.
 꼭이요.</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F17" t="inlineStr">
+      <c r="E20" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F20" t="inlineStr">
         <is>
           <t>1202,1203,1204</t>
         </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>1202</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>player</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>사담 나누기</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>1203</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>player</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>증거 구하기</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>1220</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>1204</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>player</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>대화 끝내기</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>-1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1220</v>
+        <v>1202</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>npc_catty</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>아직 아는 게 없어.</t>
+          <t>사담 나누기</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1300</v>
+        <v>1203</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>npc_phonekids</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>이 블로그 봐. 우리 마을의 이야기를 쓰고 있어.</t>
+          <t>증거 구하기</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1301</v>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>meet:npc_phonekids</t>
-        </is>
+        <v>1220</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1301</v>
+        <v>1204</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>npc_phonekids</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>글쎄, 누가 우리 마을 보물을 정리해서 올리고 있다니까?</t>
+          <t>대화 끝내기</t>
         </is>
       </c>
       <c r="E23" t="n">
         <v>-1</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>1302,1303,1304</t>
-        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1302</v>
+        <v>1220</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_catty</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>사담 나누기</t>
+          <t>아직 아는 게 없어.</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>1310</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1303</v>
+        <v>1300</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_phonekids</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>증거 구하기</t>
+          <t>이 블로그 봐. 우리 마을의 이야기를 쓰고 있어.</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>1320</v>
+        <v>1301</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>meet:npc_phonekids</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1304</v>
+        <v>1301</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_phonekids</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>대화 끝내기</t>
+          <t>글쎄, 누가 우리 마을 보물을 정리해서 올리고 있다니까?</t>
         </is>
       </c>
       <c r="E26" t="n">
         <v>-1</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>1302,1303,1304</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
+        <v>1302</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>사담 나누기</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
         <v>1310</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>npc_phonekids</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>누군지 몰라도 대단한 팬인가봐. 그렇지?</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>1302,1303,1304</t>
-        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
+        <v>1303</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>증거 구하기</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
         <v>1320</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>npc_phonekids</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>아직 아는 게 없어.</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>1301</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1400</v>
+        <v>1304</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>npc_mouse</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>찍.</t>
+          <t>대화 끝내기</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>1401</v>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>meet:npc_mouse;addNote:104</t>
-        </is>
+        <v>-1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1401</v>
+        <v>1310</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>npc_mouse</t>
+          <t>npc_phonekids</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>찍찍.</t>
+          <t>누군지 몰라도 대단한 팬인가봐. 그렇지?</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -1095,121 +1090,131 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>1402,1403,1404</t>
+          <t>1302,1303,1304</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1402</v>
+        <v>1320</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_phonekids</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>사담 나누기</t>
+          <t>아직 아는 게 없어.</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>1410</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1403</v>
+        <v>1400</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_mouse</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>증거 구하기</t>
+          <t>찍.</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>1420</v>
+        <v>1401</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>meet:npc_mouse;addNote:104</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1404</v>
+        <v>1401</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_mouse</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>대화 끝내기</t>
+          <t>찍찍.</t>
         </is>
       </c>
       <c r="E33" t="n">
         <v>-1</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>1402,1403,1404</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
+        <v>1402</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>사담 나누기</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
         <v>1410</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>npc_mouse</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>뭐? 친구??</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>1411</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>1411</v>
+        <v>1403</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>npc_mouse</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>흥! 난 그런거 필요 없어!</t>
+          <t>증거 구하기</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1412</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>1412</v>
+        <v>1404</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>npc_mouse</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>그런 사사로운 친분이 없어도 난 이미 모든 정보를 알고있다고!</t>
+          <t>대화 끝내기</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>1413</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>1413</v>
+        <v>1410</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1218,16 +1223,16 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>뭐, 사탕 가게 주인은 좋은 사람이긴 해.</t>
+          <t>뭐? 친구??</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>1401</v>
+        <v>1411</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>1420</v>
+        <v>1411</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1236,170 +1241,170 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>아직 아는 게 없어.</t>
+          <t>흥! 난 그런거 필요 없어!</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>1401</v>
+        <v>1412</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>1500</v>
+        <v>1412</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>npc_seal</t>
+          <t>npc_mouse</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>안녕하세요. 처음 뵙는 분이시네요.</t>
+          <t>그런 사사로운 친분이 없어도 난 이미 모든 정보를 알고있다고!</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1501</v>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>meet:npc_seal;addNote:105</t>
-        </is>
+        <v>1413</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>1501</v>
+        <v>1413</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>npc_seal</t>
+          <t>npc_mouse</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>저는 마을 집배원이에요.</t>
+          <t>뭐, 사탕 가게 주인은 좋은 사람이긴 해.</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>1502,1503,1504</t>
-        </is>
+        <v>1401</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>1502</v>
+        <v>1420</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_mouse</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>사담 나누기</t>
+          <t>아직 아는 게 없어.</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>1510</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>1503</v>
+        <v>1500</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_seal</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>증거 구하기</t>
+          <t>안녕하세요. 처음 뵙는 분이시네요.</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1520</v>
+        <v>1501</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>meet:npc_seal;addNote:105</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>1504</v>
+        <v>1501</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_seal</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>대화 끝내기</t>
+          <t>저는 마을 집배원이에요.</t>
         </is>
       </c>
       <c r="E43" t="n">
         <v>-1</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>1502,1503,1504</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
+        <v>1502</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>사담 나누기</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
         <v>1510</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>npc_seal</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>새로 이사왔나요? 주소를 알아야 배달할 수 있답니다.</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>1511</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>1511</v>
+        <v>1503</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>npc_seal</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>제가 모르는 얼굴... 아니 집은 없답니다.</t>
+          <t>증거 구하기</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>1590</v>
+        <v>1520</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>1520</v>
+        <v>1504</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>npc_seal</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>아직 아는 게 없어.</t>
+          <t>대화 끝내기</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>1590</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>1590</v>
+        <v>1510</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -1408,80 +1413,75 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>다른 용무가 있으신가요?</t>
+          <t>새로 이사왔나요? 주소를 알아야 배달할 수 있답니다.</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>1502,1503,1504</t>
-        </is>
+        <v>1511</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>1600</v>
+        <v>1511</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
+          <t>npc_seal</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>보물은 우리 마을의 목숨같은 존재야.</t>
+          <t>제가 모르는 얼굴... 아니 집은 없답니다.</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>1601</v>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>meet:npc_mayor;addNote:101;startQuest:1</t>
-        </is>
+        <v>1590</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1601</v>
+        <v>1520</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
+          <t>npc_seal</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>자네의 역할이 아주 중요하다는 말일세.</t>
+          <t>아직 아는 게 없어.</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>1602</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>1602</v>
+        <v>1590</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
+          <t>npc_seal</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>흠흠...</t>
+          <t>다른 용무가 있으신가요?</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>1603</v>
+        <v>-1</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>1502,1503,1504</t>
+        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1603</v>
+        <v>1600</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1490,64 +1490,66 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>아무튼! 잘 부탁한다는 뜻일세.</t>
+          <t>보물은 우리 마을의 목숨같은 존재야.</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>-1</v>
+        <v>1601</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>meet:npc_mayor;addNote:101;startQuest:1</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>9000</v>
+        <v>1601</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>narrator</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr"/>
+          <t>npc_mayor</t>
+        </is>
+      </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>12월 16일, 일요일 밤.</t>
+          <t>자네의 역할이 아주 중요하다는 말일세.</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>9001</v>
+        <v>1602</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>9001</v>
+        <v>1602</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>narrator</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr"/>
+          <t>npc_mayor</t>
+        </is>
+      </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>깨끗한 빨간 버스 한 대가 보라 마을에 도착했다.</t>
+          <t>흠흠...</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>9002</v>
+        <v>1603</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>9002</v>
+        <v>1603</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>narrator</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr"/>
+          <t>npc_mayor</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>코트에 모자를 쓴 누군가가 짐을 들고 긴 언덕길을 오른다.</t>
+          <t>아무튼! 잘 부탁한다는 뜻일세.</t>
         </is>
       </c>
       <c r="E54" t="n">
@@ -1556,76 +1558,61 @@
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>9010</v>
+        <v>9000</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>촌장</t>
+          <t>narrator</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>탐정 양반! 기다리고 있었네.</t>
+          <t>12월 16일, 일요일 밤.</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>9011</v>
+        <v>9001</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>9011</v>
+        <v>9001</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>촌장</t>
+          <t>narrator</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>지난 수요일, 12월 12일에 마을의 보물이 사라진 걸 알았지.</t>
+          <t>깨끗한 빨간 버스 한 대가 보라 마을에 도착했다.</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>9012</v>
+        <v>9002</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>9012</v>
+        <v>9002</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>촌장</t>
+          <t>narrator</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>무엇보다 범인을 찾는 게 먼저일세. 범인은... 분명 이 마을 주민이야.</t>
+          <t>코트에 모자를 쓴 누군가가 짐을 들고 긴 언덕길을 오른다.</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>9013</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>9013</v>
+        <v>9010</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -1639,72 +1626,220 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>그럼 잘 부탁하네! 난 이만 바빠서.</t>
+          <t>탐정 양반! 기다리고 있었네.</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>-1</v>
-      </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>meet:npc_mayor;addNote:101;startQuest:1</t>
-        </is>
+        <v>9011</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>9020</v>
+        <v>9011</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>narrator</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr"/>
+          <t>npc_mayor</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>촌장</t>
+        </is>
+      </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>오전 7시. 1층 간판을 뒤집었다.</t>
+          <t>지난 수요일, 12월 12일에 마을의 보물이 사라진 걸 알았지.</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>9021</v>
+        <v>9012</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>9021</v>
+        <v>9012</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>narrator</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr"/>
+          <t>npc_mayor</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>촌장</t>
+        </is>
+      </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>'탐정 사무소 오픈. 도움이 필요하다면 언제든지 방문 환영.'</t>
+          <t>무엇보다 범인을 찾는 게 먼저일세. 범인은... 분명 이 마을 주민이야.</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>9022</v>
+        <v>9013</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
+        <v>9013</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>npc_mayor</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>촌장</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>그럼 잘 부탁하네! 난 이만 바빠서.</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>meet:npc_mayor;addNote:101;startQuest:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>9020</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>오전 7시. 1층 간판을 뒤집었다.</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>9021</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>9021</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>'탐정 사무소 오픈. 도움이 필요하다면 언제든지 방문 환영.'</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
         <v>9022</v>
       </c>
-      <c r="B61" t="inlineStr">
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>9022</v>
+      </c>
+      <c r="B64" t="inlineStr">
         <is>
           <t>narrator</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>...공기가 차갑다.</t>
         </is>
       </c>
-      <c r="E61" t="n">
+      <c r="E64" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>9100</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>사무소 책상. 수첩과 서류가 가지런히 놓여 있다.</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>-1</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>9101,9102</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>9101</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>오늘 일을 수첩에 정리한다.</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>9103</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>save</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>9102</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>그만둔다.</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>9103</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>수첩을 덮었다. 잠깐 숨을 돌린다.</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
         <v>-1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(world): story gates and condition toggles
- IInteractionGate checked by RailConnector and SceneExitZone before moving
- StoryGate blocks area exits until conditions pass, shows dialogue 9200
- StoryConditionToggle switches objects by flag conditions (time slot, progress)
- Roadmap notes the expected PlazaLayout merge conflict

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Table/Excel/Dialogue.xlsx
+++ b/Table/Excel/Dialogue.xlsx
@@ -125,8 +125,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DialogueTable" displayName="DialogueTable" ref="A1:H68" headerRowCount="1">
-  <autoFilter ref="A1:H68"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DialogueTable" displayName="DialogueTable" ref="A1:H69" headerRowCount="1">
+  <autoFilter ref="A1:H69"/>
   <tableColumns count="8">
     <tableColumn id="1" name="DataId"/>
     <tableColumn id="2" name="SpeakerId"/>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1843,6 +1843,24 @@
         <v>-1</v>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>9200</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>아직 이 근처에서 알아볼 게 남은 것 같다. 수첩을 다시 확인해 보자.</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>-1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
feat(dialogue): talk menu wording and request choice from design
Choices: 사담 / 조사할 것이... (main quest active) / 부탁할 것이 있는지
(NPC has an unstarted quest this chapter) / 끝. Gumman's quest 101 now
starts from the request choice instead of the greeting. ChoiceIds max 4,
fourth button in PF_DialogueUI.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Table/Excel/Dialogue.xlsx
+++ b/Table/Excel/Dialogue.xlsx
@@ -175,8 +175,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Dialogue" displayName="Dialogue" ref="B2:I71" headerRowCount="1" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="B2:I71"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Dialogue" displayName="Dialogue" ref="B2:I73" headerRowCount="1" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="B2:I73"/>
   <tableColumns count="8">
     <tableColumn id="1" name="DataId"/>
     <tableColumn id="2" name="SpeakerId" dataDxfId="6"/>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I71"/>
+  <dimension ref="B2:I73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col width="3.125" customWidth="1" style="3" min="1" max="1"/>
@@ -822,13 +822,13 @@
       </c>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>1101,1102,1103</t>
+          <t>1101,1102,1104,1103</t>
         </is>
       </c>
       <c r="H12" s="4" t="n"/>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>meet:npc_gumman;addNote:102;startQuest:101</t>
+          <t>meet:npc_gumman;addNote:102</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,11 @@
         <v>1120</v>
       </c>
       <c r="G14" s="4" t="n"/>
-      <c r="H14" s="4" t="n"/>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>quest:1=1</t>
+        </is>
+      </c>
       <c r="I14" s="4" t="n"/>
     </row>
     <row r="15" ht="16.5" customHeight="1" s="3">
@@ -900,51 +904,51 @@
     </row>
     <row r="16" ht="16.5" customHeight="1" s="3">
       <c r="B16" s="0" t="n">
-        <v>1110</v>
-      </c>
-      <c r="C16" s="1" t="n"/>
+        <v>1104</v>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
       <c r="D16" s="4" t="n"/>
-      <c r="E16" s="1" t="n"/>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>@ui.talk_menu.request</t>
+        </is>
+      </c>
       <c r="F16" s="0" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>1111,1112,1113</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="n"/>
+        <v>1130</v>
+      </c>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>!quest:101;flag:chapter==1</t>
+        </is>
+      </c>
       <c r="I16" s="4" t="n"/>
     </row>
     <row r="17" ht="16.5" customHeight="1" s="3">
       <c r="B17" s="0" t="n">
-        <v>1111</v>
-      </c>
-      <c r="C17" s="1" t="inlineStr">
-        <is>
-          <t>npc_gumman</t>
-        </is>
-      </c>
+        <v>1110</v>
+      </c>
+      <c r="C17" s="1" t="n"/>
       <c r="D17" s="4" t="n"/>
-      <c r="E17" s="1" t="inlineStr">
-        <is>
-          <t>@dialogue.1111</t>
-        </is>
-      </c>
+      <c r="E17" s="1" t="n"/>
       <c r="F17" s="0" t="n">
         <v>-1</v>
       </c>
-      <c r="G17" s="4" t="n"/>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>flag:talk.npc_gumman&lt;=1</t>
-        </is>
-      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>1111,1112,1113</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="n"/>
       <c r="I17" s="4" t="n"/>
     </row>
     <row r="18" ht="16.5" customHeight="1" s="3">
       <c r="B18" s="0" t="n">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
@@ -954,7 +958,7 @@
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1112</t>
+          <t>@dialogue.1111</t>
         </is>
       </c>
       <c r="F18" s="0" t="n">
@@ -963,14 +967,14 @@
       <c r="G18" s="4" t="n"/>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>flag:talk.npc_gumman==2</t>
+          <t>flag:talk.npc_gumman&lt;=1</t>
         </is>
       </c>
       <c r="I18" s="4" t="n"/>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="3">
       <c r="B19" s="0" t="n">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
@@ -980,19 +984,23 @@
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1113</t>
+          <t>@dialogue.1112</t>
         </is>
       </c>
       <c r="F19" s="0" t="n">
         <v>-1</v>
       </c>
       <c r="G19" s="1" t="n"/>
-      <c r="H19" s="4" t="n"/>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>flag:talk.npc_gumman==2</t>
+        </is>
+      </c>
       <c r="I19" s="4" t="n"/>
     </row>
     <row r="20" ht="16.5" customHeight="1" s="3">
       <c r="B20" s="0" t="n">
-        <v>1120</v>
+        <v>1113</v>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
@@ -1002,11 +1010,11 @@
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.common.no_clue</t>
+          <t>@dialogue.1113</t>
         </is>
       </c>
       <c r="F20" s="0" t="n">
-        <v>1100</v>
+        <v>-1</v>
       </c>
       <c r="G20" s="4" t="n"/>
       <c r="H20" s="4" t="n"/>
@@ -1014,103 +1022,107 @@
     </row>
     <row r="21" ht="16.5" customHeight="1" s="3">
       <c r="B21" s="0" t="n">
-        <v>1200</v>
+        <v>1120</v>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>npc_catty</t>
+          <t>npc_gumman</t>
         </is>
       </c>
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1200</t>
+          <t>@dialogue.common.no_clue</t>
         </is>
       </c>
       <c r="F21" s="0" t="n">
-        <v>1201</v>
+        <v>1100</v>
       </c>
       <c r="G21" s="4" t="n"/>
       <c r="H21" s="4" t="n"/>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>meet:npc_catty</t>
-        </is>
-      </c>
+      <c r="I21" s="4" t="n"/>
     </row>
     <row r="22" ht="16.5" customHeight="1" s="3">
       <c r="B22" s="0" t="n">
-        <v>1201</v>
+        <v>1130</v>
       </c>
       <c r="C22" s="1" t="inlineStr">
         <is>
-          <t>npc_catty</t>
+          <t>npc_gumman</t>
         </is>
       </c>
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1201</t>
+          <t>@dialogue.1130</t>
         </is>
       </c>
       <c r="F22" s="0" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>1202,1203,1204</t>
-        </is>
-      </c>
+        <v>1100</v>
+      </c>
+      <c r="G22" s="4" t="n"/>
       <c r="H22" s="4" t="n"/>
-      <c r="I22" s="4" t="n"/>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>startQuest:101</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="16.5" customHeight="1" s="3">
       <c r="B23" s="0" t="n">
-        <v>1202</v>
+        <v>1200</v>
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_catty</t>
         </is>
       </c>
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="1" t="inlineStr">
         <is>
-          <t>@ui.talk_menu.chat</t>
+          <t>@dialogue.1200</t>
         </is>
       </c>
       <c r="F23" s="0" t="n">
-        <v>1200</v>
+        <v>1201</v>
       </c>
       <c r="G23" s="4" t="n"/>
       <c r="H23" s="4" t="n"/>
-      <c r="I23" s="4" t="n"/>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>meet:npc_catty</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="16.5" customHeight="1" s="3">
       <c r="B24" s="0" t="n">
-        <v>1203</v>
+        <v>1201</v>
       </c>
       <c r="C24" s="1" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_catty</t>
         </is>
       </c>
       <c r="D24" s="4" t="n"/>
       <c r="E24" s="1" t="inlineStr">
         <is>
-          <t>@ui.talk_menu.evidence</t>
+          <t>@dialogue.1201</t>
         </is>
       </c>
       <c r="F24" s="0" t="n">
-        <v>1220</v>
-      </c>
-      <c r="G24" s="4" t="n"/>
+        <v>-1</v>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>1202,1203,1204</t>
+        </is>
+      </c>
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
     </row>
     <row r="25" ht="16.5" customHeight="1" s="3">
       <c r="B25" s="0" t="n">
-        <v>1204</v>
+        <v>1202</v>
       </c>
       <c r="C25" s="1" t="inlineStr">
         <is>
@@ -1120,11 +1132,11 @@
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="1" t="inlineStr">
         <is>
-          <t>@ui.talk_menu.end</t>
+          <t>@ui.talk_menu.chat</t>
         </is>
       </c>
       <c r="F25" s="0" t="n">
-        <v>-1</v>
+        <v>1200</v>
       </c>
       <c r="G25" s="1" t="n"/>
       <c r="H25" s="4" t="n"/>
@@ -1132,125 +1144,129 @@
     </row>
     <row r="26" ht="16.5" customHeight="1" s="3">
       <c r="B26" s="0" t="n">
-        <v>1220</v>
+        <v>1203</v>
       </c>
       <c r="C26" s="1" t="inlineStr">
         <is>
-          <t>npc_catty</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.common.no_clue</t>
+          <t>@ui.talk_menu.evidence</t>
         </is>
       </c>
       <c r="F26" s="0" t="n">
-        <v>1201</v>
+        <v>1220</v>
       </c>
       <c r="G26" s="4" t="n"/>
-      <c r="H26" s="4" t="n"/>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>quest:1=1</t>
+        </is>
+      </c>
       <c r="I26" s="4" t="n"/>
     </row>
     <row r="27" ht="16.5" customHeight="1" s="3">
       <c r="B27" s="0" t="n">
-        <v>1300</v>
+        <v>1204</v>
       </c>
       <c r="C27" s="1" t="inlineStr">
         <is>
-          <t>npc_phonekids</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D27" s="4" t="n"/>
       <c r="E27" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1300</t>
+          <t>@ui.talk_menu.end</t>
         </is>
       </c>
       <c r="F27" s="0" t="n">
-        <v>1301</v>
+        <v>-1</v>
       </c>
       <c r="G27" s="4" t="n"/>
       <c r="H27" s="4" t="n"/>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>meet:npc_phonekids</t>
-        </is>
-      </c>
+      <c r="I27" s="4" t="n"/>
     </row>
     <row r="28" ht="16.5" customHeight="1" s="3">
       <c r="B28" s="0" t="n">
-        <v>1301</v>
+        <v>1220</v>
       </c>
       <c r="C28" s="1" t="inlineStr">
         <is>
-          <t>npc_phonekids</t>
+          <t>npc_catty</t>
         </is>
       </c>
       <c r="D28" s="4" t="n"/>
       <c r="E28" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1301</t>
+          <t>@dialogue.common.no_clue</t>
         </is>
       </c>
       <c r="F28" s="0" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>1302,1303,1304</t>
-        </is>
-      </c>
+        <v>1201</v>
+      </c>
+      <c r="G28" s="4" t="n"/>
       <c r="H28" s="4" t="n"/>
       <c r="I28" s="4" t="n"/>
     </row>
     <row r="29" ht="16.5" customHeight="1" s="3">
       <c r="B29" s="0" t="n">
-        <v>1302</v>
+        <v>1300</v>
       </c>
       <c r="C29" s="1" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_phonekids</t>
         </is>
       </c>
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="1" t="inlineStr">
         <is>
-          <t>@ui.talk_menu.chat</t>
+          <t>@dialogue.1300</t>
         </is>
       </c>
       <c r="F29" s="0" t="n">
-        <v>1310</v>
+        <v>1301</v>
       </c>
       <c r="G29" s="1" t="n"/>
       <c r="H29" s="4" t="n"/>
-      <c r="I29" s="4" t="n"/>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>meet:npc_phonekids</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="16.5" customHeight="1" s="3">
       <c r="B30" s="0" t="n">
-        <v>1303</v>
+        <v>1301</v>
       </c>
       <c r="C30" s="1" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_phonekids</t>
         </is>
       </c>
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="1" t="inlineStr">
         <is>
-          <t>@ui.talk_menu.evidence</t>
+          <t>@dialogue.1301</t>
         </is>
       </c>
       <c r="F30" s="0" t="n">
-        <v>1320</v>
-      </c>
-      <c r="G30" s="4" t="n"/>
+        <v>-1</v>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>1302,1303,1304</t>
+        </is>
+      </c>
       <c r="H30" s="4" t="n"/>
       <c r="I30" s="4" t="n"/>
     </row>
     <row r="31" ht="16.5" customHeight="1" s="3">
       <c r="B31" s="0" t="n">
-        <v>1304</v>
+        <v>1302</v>
       </c>
       <c r="C31" s="1" t="inlineStr">
         <is>
@@ -1260,11 +1276,11 @@
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="1" t="inlineStr">
         <is>
-          <t>@ui.talk_menu.end</t>
+          <t>@ui.talk_menu.chat</t>
         </is>
       </c>
       <c r="F31" s="0" t="n">
-        <v>-1</v>
+        <v>1310</v>
       </c>
       <c r="G31" s="4" t="n"/>
       <c r="H31" s="4" t="n"/>
@@ -1272,47 +1288,47 @@
     </row>
     <row r="32" ht="16.5" customHeight="1" s="3">
       <c r="B32" s="0" t="n">
-        <v>1310</v>
+        <v>1303</v>
       </c>
       <c r="C32" s="1" t="inlineStr">
         <is>
-          <t>npc_phonekids</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D32" s="4" t="n"/>
       <c r="E32" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1310</t>
+          <t>@ui.talk_menu.evidence</t>
         </is>
       </c>
       <c r="F32" s="0" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G32" s="1" t="inlineStr">
-        <is>
-          <t>1302,1303,1304</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="n"/>
+        <v>1320</v>
+      </c>
+      <c r="G32" s="1" t="n"/>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>quest:1=1</t>
+        </is>
+      </c>
       <c r="I32" s="4" t="n"/>
     </row>
     <row r="33" ht="16.5" customHeight="1" s="3">
       <c r="B33" s="0" t="n">
-        <v>1320</v>
+        <v>1304</v>
       </c>
       <c r="C33" s="1" t="inlineStr">
         <is>
-          <t>npc_phonekids</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.common.no_clue</t>
+          <t>@ui.talk_menu.end</t>
         </is>
       </c>
       <c r="F33" s="0" t="n">
-        <v>1301</v>
+        <v>-1</v>
       </c>
       <c r="G33" s="4" t="n"/>
       <c r="H33" s="4" t="n"/>
@@ -1320,103 +1336,107 @@
     </row>
     <row r="34" ht="16.5" customHeight="1" s="3">
       <c r="B34" s="0" t="n">
-        <v>1400</v>
+        <v>1310</v>
       </c>
       <c r="C34" s="1" t="inlineStr">
         <is>
-          <t>npc_mouse</t>
+          <t>npc_phonekids</t>
         </is>
       </c>
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1400</t>
+          <t>@dialogue.1310</t>
         </is>
       </c>
       <c r="F34" s="0" t="n">
-        <v>1401</v>
-      </c>
-      <c r="G34" s="4" t="n"/>
+        <v>-1</v>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>1302,1303,1304</t>
+        </is>
+      </c>
       <c r="H34" s="4" t="n"/>
-      <c r="I34" s="4" t="inlineStr">
-        <is>
-          <t>meet:npc_mouse;addNote:104</t>
-        </is>
-      </c>
+      <c r="I34" s="4" t="n"/>
     </row>
     <row r="35" ht="16.5" customHeight="1" s="3">
       <c r="B35" s="0" t="n">
-        <v>1401</v>
+        <v>1320</v>
       </c>
       <c r="C35" s="1" t="inlineStr">
         <is>
-          <t>npc_mouse</t>
+          <t>npc_phonekids</t>
         </is>
       </c>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1401</t>
+          <t>@dialogue.common.no_clue</t>
         </is>
       </c>
       <c r="F35" s="0" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>1402,1403,1404</t>
-        </is>
-      </c>
+        <v>1301</v>
+      </c>
+      <c r="G35" s="4" t="n"/>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
     </row>
     <row r="36" ht="16.5" customHeight="1" s="3">
       <c r="B36" s="0" t="n">
-        <v>1402</v>
+        <v>1400</v>
       </c>
       <c r="C36" s="1" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_mouse</t>
         </is>
       </c>
       <c r="D36" s="4" t="n"/>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>@ui.talk_menu.chat</t>
+          <t>@dialogue.1400</t>
         </is>
       </c>
       <c r="F36" s="0" t="n">
-        <v>1410</v>
+        <v>1401</v>
       </c>
       <c r="G36" s="4" t="n"/>
       <c r="H36" s="4" t="n"/>
-      <c r="I36" s="4" t="n"/>
+      <c r="I36" s="4" t="inlineStr">
+        <is>
+          <t>meet:npc_mouse;addNote:104</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="16.5" customHeight="1" s="3">
       <c r="B37" s="0" t="n">
-        <v>1403</v>
+        <v>1401</v>
       </c>
       <c r="C37" s="1" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_mouse</t>
         </is>
       </c>
       <c r="D37" s="4" t="n"/>
       <c r="E37" s="1" t="inlineStr">
         <is>
-          <t>@ui.talk_menu.evidence</t>
+          <t>@dialogue.1401</t>
         </is>
       </c>
       <c r="F37" s="0" t="n">
-        <v>1420</v>
-      </c>
-      <c r="G37" s="4" t="n"/>
+        <v>-1</v>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>1402,1403,1404</t>
+        </is>
+      </c>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
     </row>
     <row r="38" ht="16.5" customHeight="1" s="3">
       <c r="B38" s="0" t="n">
-        <v>1404</v>
+        <v>1402</v>
       </c>
       <c r="C38" s="1" t="inlineStr">
         <is>
@@ -1426,11 +1446,11 @@
       <c r="D38" s="4" t="n"/>
       <c r="E38" s="1" t="inlineStr">
         <is>
-          <t>@ui.talk_menu.end</t>
+          <t>@ui.talk_menu.chat</t>
         </is>
       </c>
       <c r="F38" s="0" t="n">
-        <v>-1</v>
+        <v>1410</v>
       </c>
       <c r="G38" s="4" t="n"/>
       <c r="H38" s="4" t="n"/>
@@ -1438,43 +1458,47 @@
     </row>
     <row r="39" ht="16.5" customHeight="1" s="3">
       <c r="B39" s="0" t="n">
-        <v>1410</v>
+        <v>1403</v>
       </c>
       <c r="C39" s="1" t="inlineStr">
         <is>
-          <t>npc_mouse</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D39" s="4" t="n"/>
       <c r="E39" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1410</t>
+          <t>@ui.talk_menu.evidence</t>
         </is>
       </c>
       <c r="F39" s="0" t="n">
-        <v>1411</v>
+        <v>1420</v>
       </c>
       <c r="G39" s="4" t="n"/>
-      <c r="H39" s="4" t="n"/>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>quest:1=1</t>
+        </is>
+      </c>
       <c r="I39" s="4" t="n"/>
     </row>
     <row r="40" ht="16.5" customHeight="1" s="3">
       <c r="B40" s="0" t="n">
-        <v>1411</v>
+        <v>1404</v>
       </c>
       <c r="C40" s="1" t="inlineStr">
         <is>
-          <t>npc_mouse</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D40" s="4" t="n"/>
       <c r="E40" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1411</t>
+          <t>@ui.talk_menu.end</t>
         </is>
       </c>
       <c r="F40" s="0" t="n">
-        <v>1412</v>
+        <v>-1</v>
       </c>
       <c r="G40" s="4" t="n"/>
       <c r="H40" s="4" t="n"/>
@@ -1482,7 +1506,7 @@
     </row>
     <row r="41" ht="16.5" customHeight="1" s="3">
       <c r="B41" s="0" t="n">
-        <v>1412</v>
+        <v>1410</v>
       </c>
       <c r="C41" s="1" t="inlineStr">
         <is>
@@ -1492,11 +1516,11 @@
       <c r="D41" s="4" t="n"/>
       <c r="E41" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1412</t>
+          <t>@dialogue.1410</t>
         </is>
       </c>
       <c r="F41" s="0" t="n">
-        <v>1413</v>
+        <v>1411</v>
       </c>
       <c r="G41" s="4" t="n"/>
       <c r="H41" s="4" t="n"/>
@@ -1504,7 +1528,7 @@
     </row>
     <row r="42" ht="16.5" customHeight="1" s="3">
       <c r="B42" s="0" t="n">
-        <v>1413</v>
+        <v>1411</v>
       </c>
       <c r="C42" s="1" t="inlineStr">
         <is>
@@ -1514,11 +1538,11 @@
       <c r="D42" s="4" t="n"/>
       <c r="E42" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1413</t>
+          <t>@dialogue.1411</t>
         </is>
       </c>
       <c r="F42" s="0" t="n">
-        <v>1401</v>
+        <v>1412</v>
       </c>
       <c r="G42" s="1" t="n"/>
       <c r="H42" s="4" t="n"/>
@@ -1526,7 +1550,7 @@
     </row>
     <row r="43" ht="16.5" customHeight="1" s="3">
       <c r="B43" s="0" t="n">
-        <v>1420</v>
+        <v>1412</v>
       </c>
       <c r="C43" s="1" t="inlineStr">
         <is>
@@ -1536,11 +1560,11 @@
       <c r="D43" s="4" t="n"/>
       <c r="E43" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.common.no_clue</t>
+          <t>@dialogue.1412</t>
         </is>
       </c>
       <c r="F43" s="0" t="n">
-        <v>1401</v>
+        <v>1413</v>
       </c>
       <c r="G43" s="4" t="n"/>
       <c r="H43" s="4" t="n"/>
@@ -1548,103 +1572,103 @@
     </row>
     <row r="44" ht="16.5" customHeight="1" s="3">
       <c r="B44" s="0" t="n">
-        <v>1500</v>
+        <v>1413</v>
       </c>
       <c r="C44" s="1" t="inlineStr">
         <is>
-          <t>npc_seal</t>
+          <t>npc_mouse</t>
         </is>
       </c>
       <c r="D44" s="4" t="n"/>
       <c r="E44" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1500</t>
+          <t>@dialogue.1413</t>
         </is>
       </c>
       <c r="F44" s="0" t="n">
-        <v>1501</v>
+        <v>1401</v>
       </c>
       <c r="G44" s="4" t="n"/>
       <c r="H44" s="4" t="n"/>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>meet:npc_seal;addNote:105</t>
-        </is>
-      </c>
+      <c r="I44" s="4" t="n"/>
     </row>
     <row r="45" ht="16.5" customHeight="1" s="3">
       <c r="B45" s="0" t="n">
-        <v>1501</v>
+        <v>1420</v>
       </c>
       <c r="C45" s="1" t="inlineStr">
         <is>
-          <t>npc_seal</t>
+          <t>npc_mouse</t>
         </is>
       </c>
       <c r="D45" s="4" t="n"/>
       <c r="E45" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1501</t>
+          <t>@dialogue.common.no_clue</t>
         </is>
       </c>
       <c r="F45" s="0" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>1502,1503,1504</t>
-        </is>
-      </c>
+        <v>1401</v>
+      </c>
+      <c r="G45" s="4" t="n"/>
       <c r="H45" s="4" t="n"/>
       <c r="I45" s="4" t="n"/>
     </row>
     <row r="46" ht="16.5" customHeight="1" s="3">
       <c r="B46" s="0" t="n">
-        <v>1502</v>
+        <v>1500</v>
       </c>
       <c r="C46" s="1" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_seal</t>
         </is>
       </c>
       <c r="D46" s="4" t="n"/>
       <c r="E46" s="1" t="inlineStr">
         <is>
-          <t>@ui.talk_menu.chat</t>
+          <t>@dialogue.1500</t>
         </is>
       </c>
       <c r="F46" s="0" t="n">
-        <v>1510</v>
+        <v>1501</v>
       </c>
       <c r="G46" s="4" t="n"/>
       <c r="H46" s="4" t="n"/>
-      <c r="I46" s="4" t="n"/>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>meet:npc_seal;addNote:105</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="16.5" customHeight="1" s="3">
       <c r="B47" s="0" t="n">
-        <v>1503</v>
+        <v>1501</v>
       </c>
       <c r="C47" s="1" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>npc_seal</t>
         </is>
       </c>
       <c r="D47" s="4" t="n"/>
       <c r="E47" s="1" t="inlineStr">
         <is>
-          <t>@ui.talk_menu.evidence</t>
+          <t>@dialogue.1501</t>
         </is>
       </c>
       <c r="F47" s="0" t="n">
-        <v>1520</v>
-      </c>
-      <c r="G47" s="4" t="n"/>
+        <v>-1</v>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>1502,1503,1504</t>
+        </is>
+      </c>
       <c r="H47" s="4" t="n"/>
       <c r="I47" s="4" t="n"/>
     </row>
     <row r="48" ht="16.5" customHeight="1" s="3">
       <c r="B48" s="0" t="n">
-        <v>1504</v>
+        <v>1502</v>
       </c>
       <c r="C48" s="1" t="inlineStr">
         <is>
@@ -1654,11 +1678,11 @@
       <c r="D48" s="4" t="n"/>
       <c r="E48" s="1" t="inlineStr">
         <is>
-          <t>@ui.talk_menu.end</t>
+          <t>@ui.talk_menu.chat</t>
         </is>
       </c>
       <c r="F48" s="0" t="n">
-        <v>-1</v>
+        <v>1510</v>
       </c>
       <c r="G48" s="4" t="n"/>
       <c r="H48" s="4" t="n"/>
@@ -1666,43 +1690,47 @@
     </row>
     <row r="49" ht="16.5" customHeight="1" s="3">
       <c r="B49" s="0" t="n">
-        <v>1510</v>
+        <v>1503</v>
       </c>
       <c r="C49" s="1" t="inlineStr">
         <is>
-          <t>npc_seal</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D49" s="4" t="n"/>
       <c r="E49" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1510</t>
+          <t>@ui.talk_menu.evidence</t>
         </is>
       </c>
       <c r="F49" s="0" t="n">
-        <v>1511</v>
+        <v>1520</v>
       </c>
       <c r="G49" s="1" t="n"/>
-      <c r="H49" s="4" t="n"/>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>quest:1=1</t>
+        </is>
+      </c>
       <c r="I49" s="4" t="n"/>
     </row>
     <row r="50" ht="16.5" customHeight="1" s="3">
       <c r="B50" s="0" t="n">
-        <v>1511</v>
+        <v>1504</v>
       </c>
       <c r="C50" s="1" t="inlineStr">
         <is>
-          <t>npc_seal</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D50" s="4" t="n"/>
       <c r="E50" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1511</t>
+          <t>@ui.talk_menu.end</t>
         </is>
       </c>
       <c r="F50" s="0" t="n">
-        <v>1590</v>
+        <v>-1</v>
       </c>
       <c r="G50" s="4" t="n"/>
       <c r="H50" s="4" t="n"/>
@@ -1710,7 +1738,7 @@
     </row>
     <row r="51" ht="16.5" customHeight="1" s="3">
       <c r="B51" s="0" t="n">
-        <v>1520</v>
+        <v>1510</v>
       </c>
       <c r="C51" s="1" t="inlineStr">
         <is>
@@ -1720,11 +1748,11 @@
       <c r="D51" s="4" t="n"/>
       <c r="E51" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.common.no_clue</t>
+          <t>@dialogue.1510</t>
         </is>
       </c>
       <c r="F51" s="0" t="n">
-        <v>1590</v>
+        <v>1511</v>
       </c>
       <c r="G51" s="4" t="n"/>
       <c r="H51" s="4" t="n"/>
@@ -1732,7 +1760,7 @@
     </row>
     <row r="52" ht="16.5" customHeight="1" s="3">
       <c r="B52" s="0" t="n">
-        <v>1590</v>
+        <v>1511</v>
       </c>
       <c r="C52" s="1" t="inlineStr">
         <is>
@@ -1742,71 +1770,67 @@
       <c r="D52" s="4" t="n"/>
       <c r="E52" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1590</t>
+          <t>@dialogue.1511</t>
         </is>
       </c>
       <c r="F52" s="0" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G52" s="4" t="inlineStr">
-        <is>
-          <t>1502,1503,1504</t>
-        </is>
-      </c>
+        <v>1590</v>
+      </c>
+      <c r="G52" s="4" t="n"/>
       <c r="H52" s="4" t="n"/>
       <c r="I52" s="4" t="n"/>
     </row>
     <row r="53" ht="16.5" customHeight="1" s="3">
       <c r="B53" s="0" t="n">
-        <v>1600</v>
+        <v>1520</v>
       </c>
       <c r="C53" s="1" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
+          <t>npc_seal</t>
         </is>
       </c>
       <c r="D53" s="4" t="n"/>
       <c r="E53" s="1" t="inlineStr">
         <is>
-          <t>@dialogue.1600</t>
+          <t>@dialogue.common.no_clue</t>
         </is>
       </c>
       <c r="F53" s="0" t="n">
-        <v>1601</v>
+        <v>1590</v>
       </c>
       <c r="G53" s="4" t="n"/>
       <c r="H53" s="4" t="n"/>
-      <c r="I53" s="4" t="inlineStr">
-        <is>
-          <t>meet:npc_mayor;addNote:101;startQuest:1</t>
-        </is>
-      </c>
+      <c r="I53" s="4" t="n"/>
     </row>
     <row r="54">
-      <c r="B54" t="n">
-        <v>1601</v>
+      <c r="B54" s="0" t="n">
+        <v>1590</v>
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
+          <t>npc_seal</t>
         </is>
       </c>
       <c r="D54" s="4" t="n"/>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.1601</t>
-        </is>
-      </c>
-      <c r="F54" t="n">
-        <v>1602</v>
-      </c>
-      <c r="G54" s="4" t="n"/>
+          <t>@dialogue.1590</t>
+        </is>
+      </c>
+      <c r="F54" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>1502,1503,1504</t>
+        </is>
+      </c>
       <c r="H54" s="4" t="n"/>
       <c r="I54" s="4" t="n"/>
     </row>
     <row r="55">
-      <c r="B55" t="n">
-        <v>1602</v>
+      <c r="B55" s="0" t="n">
+        <v>1600</v>
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
@@ -1816,19 +1840,23 @@
       <c r="D55" s="4" t="n"/>
       <c r="E55" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.1602</t>
-        </is>
-      </c>
-      <c r="F55" t="n">
-        <v>1603</v>
+          <t>@dialogue.1600</t>
+        </is>
+      </c>
+      <c r="F55" s="0" t="n">
+        <v>1601</v>
       </c>
       <c r="G55" s="4" t="n"/>
       <c r="H55" s="4" t="n"/>
-      <c r="I55" s="4" t="n"/>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>meet:npc_mayor;addNote:101;startQuest:1</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="B56" t="n">
-        <v>1603</v>
+      <c r="B56" s="0" t="n">
+        <v>1601</v>
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
@@ -1838,63 +1866,63 @@
       <c r="D56" s="4" t="n"/>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.1603</t>
-        </is>
-      </c>
-      <c r="F56" t="n">
-        <v>-1</v>
+          <t>@dialogue.1601</t>
+        </is>
+      </c>
+      <c r="F56" s="0" t="n">
+        <v>1602</v>
       </c>
       <c r="G56" s="4" t="n"/>
       <c r="H56" s="4" t="n"/>
       <c r="I56" s="4" t="n"/>
     </row>
     <row r="57">
-      <c r="B57" t="n">
-        <v>9000</v>
+      <c r="B57" s="0" t="n">
+        <v>1602</v>
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
+          <t>npc_mayor</t>
         </is>
       </c>
       <c r="D57" s="4" t="n"/>
       <c r="E57" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9000</t>
-        </is>
-      </c>
-      <c r="F57" t="n">
-        <v>9001</v>
+          <t>@dialogue.1602</t>
+        </is>
+      </c>
+      <c r="F57" s="0" t="n">
+        <v>1603</v>
       </c>
       <c r="G57" s="4" t="n"/>
       <c r="H57" s="4" t="n"/>
       <c r="I57" s="4" t="n"/>
     </row>
     <row r="58">
-      <c r="B58" t="n">
-        <v>9001</v>
+      <c r="B58" s="0" t="n">
+        <v>1603</v>
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
+          <t>npc_mayor</t>
         </is>
       </c>
       <c r="D58" s="4" t="n"/>
       <c r="E58" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9001</t>
-        </is>
-      </c>
-      <c r="F58" t="n">
-        <v>9002</v>
+          <t>@dialogue.1603</t>
+        </is>
+      </c>
+      <c r="F58" s="0" t="n">
+        <v>-1</v>
       </c>
       <c r="G58" s="4" t="n"/>
       <c r="H58" s="4" t="n"/>
       <c r="I58" s="4" t="n"/>
     </row>
     <row r="59">
-      <c r="B59" t="n">
-        <v>9002</v>
+      <c r="B59" s="0" t="n">
+        <v>9000</v>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
@@ -1904,71 +1932,63 @@
       <c r="D59" s="4" t="n"/>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9002</t>
-        </is>
-      </c>
-      <c r="F59" t="n">
-        <v>-1</v>
+          <t>@dialogue.9000</t>
+        </is>
+      </c>
+      <c r="F59" s="0" t="n">
+        <v>9001</v>
       </c>
       <c r="G59" s="4" t="n"/>
       <c r="H59" s="4" t="n"/>
       <c r="I59" s="4" t="n"/>
     </row>
     <row r="60">
-      <c r="B60" t="n">
-        <v>9010</v>
+      <c r="B60" s="0" t="n">
+        <v>9001</v>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
-        </is>
-      </c>
-      <c r="D60" s="4" t="inlineStr">
-        <is>
-          <t>촌장</t>
-        </is>
-      </c>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="n"/>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9010</t>
-        </is>
-      </c>
-      <c r="F60" t="n">
-        <v>9011</v>
+          <t>@dialogue.9001</t>
+        </is>
+      </c>
+      <c r="F60" s="0" t="n">
+        <v>9002</v>
       </c>
       <c r="G60" s="4" t="n"/>
       <c r="H60" s="4" t="n"/>
       <c r="I60" s="4" t="n"/>
     </row>
     <row r="61">
-      <c r="B61" t="n">
-        <v>9011</v>
+      <c r="B61" s="0" t="n">
+        <v>9002</v>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
-        </is>
-      </c>
-      <c r="D61" s="4" t="inlineStr">
-        <is>
-          <t>촌장</t>
-        </is>
-      </c>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="n"/>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9011</t>
-        </is>
-      </c>
-      <c r="F61" t="n">
-        <v>9012</v>
+          <t>@dialogue.9002</t>
+        </is>
+      </c>
+      <c r="F61" s="0" t="n">
+        <v>-1</v>
       </c>
       <c r="G61" s="4" t="n"/>
       <c r="H61" s="4" t="n"/>
       <c r="I61" s="4" t="n"/>
     </row>
     <row r="62">
-      <c r="B62" t="n">
-        <v>9012</v>
+      <c r="B62" s="0" t="n">
+        <v>9010</v>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
@@ -1982,19 +2002,19 @@
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9012</t>
-        </is>
-      </c>
-      <c r="F62" t="n">
-        <v>9013</v>
+          <t>@dialogue.9010</t>
+        </is>
+      </c>
+      <c r="F62" s="0" t="n">
+        <v>9011</v>
       </c>
       <c r="G62" s="4" t="n"/>
       <c r="H62" s="4" t="n"/>
       <c r="I62" s="4" t="n"/>
     </row>
     <row r="63">
-      <c r="B63" t="n">
-        <v>9013</v>
+      <c r="B63" s="0" t="n">
+        <v>9011</v>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
@@ -2008,67 +2028,75 @@
       </c>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9013</t>
-        </is>
-      </c>
-      <c r="F63" t="n">
-        <v>-1</v>
+          <t>@dialogue.9011</t>
+        </is>
+      </c>
+      <c r="F63" s="0" t="n">
+        <v>9012</v>
       </c>
       <c r="G63" s="4" t="n"/>
       <c r="H63" s="4" t="n"/>
-      <c r="I63" s="4" t="inlineStr">
-        <is>
-          <t>meet:npc_mayor;addNote:101;startQuest:1</t>
-        </is>
-      </c>
+      <c r="I63" s="4" t="n"/>
     </row>
     <row r="64">
-      <c r="B64" t="n">
-        <v>9020</v>
+      <c r="B64" s="0" t="n">
+        <v>9012</v>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
-        </is>
-      </c>
-      <c r="D64" s="4" t="n"/>
+          <t>npc_mayor</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>촌장</t>
+        </is>
+      </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9020</t>
-        </is>
-      </c>
-      <c r="F64" t="n">
-        <v>9021</v>
+          <t>@dialogue.9012</t>
+        </is>
+      </c>
+      <c r="F64" s="0" t="n">
+        <v>9013</v>
       </c>
       <c r="G64" s="4" t="n"/>
       <c r="H64" s="4" t="n"/>
       <c r="I64" s="4" t="n"/>
     </row>
     <row r="65">
-      <c r="B65" t="n">
-        <v>9021</v>
+      <c r="B65" s="0" t="n">
+        <v>9013</v>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="n"/>
+          <t>npc_mayor</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>촌장</t>
+        </is>
+      </c>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9021</t>
-        </is>
-      </c>
-      <c r="F65" t="n">
-        <v>9022</v>
+          <t>@dialogue.9013</t>
+        </is>
+      </c>
+      <c r="F65" s="0" t="n">
+        <v>-1</v>
       </c>
       <c r="G65" s="4" t="n"/>
       <c r="H65" s="4" t="n"/>
-      <c r="I65" s="4" t="n"/>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>meet:npc_mayor;addNote:101;startQuest:1</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="B66" t="n">
-        <v>9022</v>
+      <c r="B66" s="0" t="n">
+        <v>9020</v>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
@@ -2078,19 +2106,19 @@
       <c r="D66" s="4" t="n"/>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9022</t>
-        </is>
-      </c>
-      <c r="F66" t="n">
-        <v>-1</v>
+          <t>@dialogue.9020</t>
+        </is>
+      </c>
+      <c r="F66" s="0" t="n">
+        <v>9021</v>
       </c>
       <c r="G66" s="4" t="n"/>
       <c r="H66" s="4" t="n"/>
       <c r="I66" s="4" t="n"/>
     </row>
     <row r="67">
-      <c r="B67" t="n">
-        <v>9100</v>
+      <c r="B67" s="0" t="n">
+        <v>9021</v>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
@@ -2100,111 +2128,155 @@
       <c r="D67" s="4" t="n"/>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9100</t>
-        </is>
-      </c>
-      <c r="F67" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G67" s="4" t="inlineStr">
-        <is>
-          <t>9101,9102</t>
-        </is>
-      </c>
+          <t>@dialogue.9021</t>
+        </is>
+      </c>
+      <c r="F67" s="0" t="n">
+        <v>9022</v>
+      </c>
+      <c r="G67" s="4" t="n"/>
       <c r="H67" s="4" t="n"/>
       <c r="I67" s="4" t="n"/>
     </row>
     <row r="68">
-      <c r="B68" t="n">
-        <v>9101</v>
+      <c r="B68" s="0" t="n">
+        <v>9022</v>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>narrator</t>
         </is>
       </c>
       <c r="D68" s="4" t="n"/>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9101</t>
-        </is>
-      </c>
-      <c r="F68" t="n">
-        <v>9103</v>
+          <t>@dialogue.9022</t>
+        </is>
+      </c>
+      <c r="F68" s="0" t="n">
+        <v>-1</v>
       </c>
       <c r="G68" s="4" t="n"/>
       <c r="H68" s="4" t="n"/>
-      <c r="I68" s="4" t="inlineStr">
-        <is>
-          <t>save</t>
-        </is>
-      </c>
+      <c r="I68" s="4" t="n"/>
     </row>
     <row r="69">
-      <c r="B69" t="n">
-        <v>9102</v>
+      <c r="B69" s="0" t="n">
+        <v>9100</v>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>player</t>
+          <t>narrator</t>
         </is>
       </c>
       <c r="D69" s="4" t="n"/>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9102</t>
-        </is>
-      </c>
-      <c r="F69" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G69" s="4" t="n"/>
+          <t>@dialogue.9100</t>
+        </is>
+      </c>
+      <c r="F69" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>9101,9102</t>
+        </is>
+      </c>
       <c r="H69" s="4" t="n"/>
       <c r="I69" s="4" t="n"/>
     </row>
     <row r="70">
-      <c r="B70" t="n">
-        <v>9103</v>
+      <c r="B70" s="0" t="n">
+        <v>9101</v>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D70" s="4" t="n"/>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9103</t>
-        </is>
-      </c>
-      <c r="F70" t="n">
-        <v>-1</v>
+          <t>@dialogue.9101</t>
+        </is>
+      </c>
+      <c r="F70" s="0" t="n">
+        <v>9103</v>
       </c>
       <c r="G70" s="4" t="n"/>
       <c r="H70" s="4" t="n"/>
-      <c r="I70" s="4" t="n"/>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>save</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="B71" t="n">
-        <v>9200</v>
+      <c r="B71" s="0" t="n">
+        <v>9102</v>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D71" s="4" t="n"/>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9200</t>
-        </is>
-      </c>
-      <c r="F71" t="n">
+          <t>@dialogue.9102</t>
+        </is>
+      </c>
+      <c r="F71" s="0" t="n">
         <v>-1</v>
       </c>
       <c r="G71" s="4" t="n"/>
       <c r="H71" s="4" t="n"/>
       <c r="I71" s="4" t="n"/>
+    </row>
+    <row r="72">
+      <c r="B72" s="0" t="n">
+        <v>9103</v>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="n"/>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9103</t>
+        </is>
+      </c>
+      <c r="F72" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G72" s="4" t="n"/>
+      <c r="H72" s="4" t="n"/>
+      <c r="I72" s="4" t="n"/>
+    </row>
+    <row r="73">
+      <c r="B73" s="0" t="n">
+        <v>9200</v>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="n"/>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9200</t>
+        </is>
+      </c>
+      <c r="F73" s="0" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G73" s="4" t="n"/>
+      <c r="H73" s="4" t="n"/>
+      <c r="I73" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(dialogue): placeholder talk menus for quest givers 102 and 103
npc_ele (1700s, quest 103) and npc_jumpropekid (1800s, quest 102) follow
the gumman pattern with "테스트 문구" text. NPCs are not placed yet.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Table/Excel/Dialogue.xlsx
+++ b/Table/Excel/Dialogue.xlsx
@@ -175,8 +175,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Dialogue" displayName="Dialogue" ref="B2:I73" headerRowCount="1" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="B2:I73"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Dialogue" displayName="Dialogue" ref="B2:I89" headerRowCount="1" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="B2:I89"/>
   <tableColumns count="8">
     <tableColumn id="1" name="DataId"/>
     <tableColumn id="2" name="SpeakerId" dataDxfId="6"/>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I73"/>
+  <dimension ref="B2:I89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" customHeight="1"/>
   <cols>
     <col width="3.125" customWidth="1" style="3" min="1" max="1"/>
@@ -1922,43 +1922,51 @@
     </row>
     <row r="59">
       <c r="B59" s="0" t="n">
-        <v>9000</v>
+        <v>1700</v>
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
+          <t>npc_ele</t>
         </is>
       </c>
       <c r="D59" s="4" t="n"/>
       <c r="E59" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9000</t>
+          <t>@dialogue.1700</t>
         </is>
       </c>
       <c r="F59" s="0" t="n">
-        <v>9001</v>
-      </c>
-      <c r="G59" s="4" t="n"/>
+        <v>-1</v>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>1701,1702,1703,1704</t>
+        </is>
+      </c>
       <c r="H59" s="4" t="n"/>
-      <c r="I59" s="4" t="n"/>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>meet:npc_ele</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="0" t="n">
-        <v>9001</v>
+        <v>1701</v>
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D60" s="4" t="n"/>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9001</t>
+          <t>@ui.talk_menu.chat</t>
         </is>
       </c>
       <c r="F60" s="0" t="n">
-        <v>9002</v>
+        <v>1710</v>
       </c>
       <c r="G60" s="4" t="n"/>
       <c r="H60" s="4" t="n"/>
@@ -1966,73 +1974,73 @@
     </row>
     <row r="61">
       <c r="B61" s="0" t="n">
-        <v>9002</v>
+        <v>1702</v>
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D61" s="4" t="n"/>
       <c r="E61" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9002</t>
+          <t>@ui.talk_menu.evidence</t>
         </is>
       </c>
       <c r="F61" s="0" t="n">
-        <v>-1</v>
+        <v>1720</v>
       </c>
       <c r="G61" s="4" t="n"/>
-      <c r="H61" s="4" t="n"/>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>quest:1=1</t>
+        </is>
+      </c>
       <c r="I61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="B62" s="0" t="n">
-        <v>9010</v>
+        <v>1703</v>
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
-        </is>
-      </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>촌장</t>
-        </is>
-      </c>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="n"/>
       <c r="E62" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9010</t>
+          <t>@ui.talk_menu.request</t>
         </is>
       </c>
       <c r="F62" s="0" t="n">
-        <v>9011</v>
+        <v>1730</v>
       </c>
       <c r="G62" s="4" t="n"/>
-      <c r="H62" s="4" t="n"/>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>!quest:103;flag:chapter==1</t>
+        </is>
+      </c>
       <c r="I62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="B63" s="0" t="n">
-        <v>9011</v>
+        <v>1704</v>
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
-        </is>
-      </c>
-      <c r="D63" s="4" t="inlineStr">
-        <is>
-          <t>촌장</t>
-        </is>
-      </c>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="n"/>
       <c r="E63" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9011</t>
+          <t>@ui.talk_menu.end</t>
         </is>
       </c>
       <c r="F63" s="0" t="n">
-        <v>9012</v>
+        <v>-1</v>
       </c>
       <c r="G63" s="4" t="n"/>
       <c r="H63" s="4" t="n"/>
@@ -2040,25 +2048,21 @@
     </row>
     <row r="64">
       <c r="B64" s="0" t="n">
-        <v>9012</v>
+        <v>1710</v>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
-        </is>
-      </c>
-      <c r="D64" s="4" t="inlineStr">
-        <is>
-          <t>촌장</t>
-        </is>
-      </c>
+          <t>npc_ele</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="n"/>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9012</t>
+          <t>@dialogue.1710</t>
         </is>
       </c>
       <c r="F64" s="0" t="n">
-        <v>9013</v>
+        <v>1700</v>
       </c>
       <c r="G64" s="4" t="n"/>
       <c r="H64" s="4" t="n"/>
@@ -2066,95 +2070,99 @@
     </row>
     <row r="65">
       <c r="B65" s="0" t="n">
-        <v>9013</v>
+        <v>1720</v>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>npc_mayor</t>
-        </is>
-      </c>
-      <c r="D65" s="4" t="inlineStr">
-        <is>
-          <t>촌장</t>
-        </is>
-      </c>
+          <t>npc_ele</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="n"/>
       <c r="E65" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9013</t>
+          <t>@dialogue.common.no_clue</t>
         </is>
       </c>
       <c r="F65" s="0" t="n">
-        <v>-1</v>
+        <v>1700</v>
       </c>
       <c r="G65" s="4" t="n"/>
       <c r="H65" s="4" t="n"/>
-      <c r="I65" s="4" t="inlineStr">
-        <is>
-          <t>meet:npc_mayor;addNote:101;startQuest:1</t>
-        </is>
-      </c>
+      <c r="I65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="B66" s="0" t="n">
-        <v>9020</v>
+        <v>1730</v>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
+          <t>npc_ele</t>
         </is>
       </c>
       <c r="D66" s="4" t="n"/>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9020</t>
+          <t>@dialogue.1730</t>
         </is>
       </c>
       <c r="F66" s="0" t="n">
-        <v>9021</v>
+        <v>1700</v>
       </c>
       <c r="G66" s="4" t="n"/>
       <c r="H66" s="4" t="n"/>
-      <c r="I66" s="4" t="n"/>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>startQuest:103</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="B67" s="0" t="n">
-        <v>9021</v>
+        <v>1800</v>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
+          <t>npc_jumpropekid</t>
         </is>
       </c>
       <c r="D67" s="4" t="n"/>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9021</t>
+          <t>@dialogue.1800</t>
         </is>
       </c>
       <c r="F67" s="0" t="n">
-        <v>9022</v>
-      </c>
-      <c r="G67" s="4" t="n"/>
+        <v>-1</v>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>1801,1802,1803,1804</t>
+        </is>
+      </c>
       <c r="H67" s="4" t="n"/>
-      <c r="I67" s="4" t="n"/>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>meet:npc_jumpropekid</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="B68" s="0" t="n">
-        <v>9022</v>
+        <v>1801</v>
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D68" s="4" t="n"/>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9022</t>
+          <t>@ui.talk_menu.chat</t>
         </is>
       </c>
       <c r="F68" s="0" t="n">
-        <v>-1</v>
+        <v>1810</v>
       </c>
       <c r="G68" s="4" t="n"/>
       <c r="H68" s="4" t="n"/>
@@ -2162,33 +2170,33 @@
     </row>
     <row r="69">
       <c r="B69" s="0" t="n">
-        <v>9100</v>
+        <v>1802</v>
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
+          <t>player</t>
         </is>
       </c>
       <c r="D69" s="4" t="n"/>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9100</t>
+          <t>@ui.talk_menu.evidence</t>
         </is>
       </c>
       <c r="F69" s="0" t="n">
-        <v>-1</v>
-      </c>
-      <c r="G69" s="4" t="inlineStr">
-        <is>
-          <t>9101,9102</t>
-        </is>
-      </c>
-      <c r="H69" s="4" t="n"/>
+        <v>1820</v>
+      </c>
+      <c r="G69" s="4" t="n"/>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>quest:1=1</t>
+        </is>
+      </c>
       <c r="I69" s="4" t="n"/>
     </row>
     <row r="70">
       <c r="B70" s="0" t="n">
-        <v>9101</v>
+        <v>1803</v>
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
@@ -2198,23 +2206,23 @@
       <c r="D70" s="4" t="n"/>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9101</t>
+          <t>@ui.talk_menu.request</t>
         </is>
       </c>
       <c r="F70" s="0" t="n">
-        <v>9103</v>
+        <v>1830</v>
       </c>
       <c r="G70" s="4" t="n"/>
-      <c r="H70" s="4" t="n"/>
-      <c r="I70" s="4" t="inlineStr">
-        <is>
-          <t>save</t>
-        </is>
-      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>!quest:102;flag:chapter==1</t>
+        </is>
+      </c>
+      <c r="I70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="B71" s="0" t="n">
-        <v>9102</v>
+        <v>1804</v>
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
@@ -2224,7 +2232,7 @@
       <c r="D71" s="4" t="n"/>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9102</t>
+          <t>@ui.talk_menu.end</t>
         </is>
       </c>
       <c r="F71" s="0" t="n">
@@ -2236,21 +2244,21 @@
     </row>
     <row r="72">
       <c r="B72" s="0" t="n">
-        <v>9103</v>
+        <v>1810</v>
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
+          <t>npc_jumpropekid</t>
         </is>
       </c>
       <c r="D72" s="4" t="n"/>
       <c r="E72" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9103</t>
+          <t>@dialogue.1810</t>
         </is>
       </c>
       <c r="F72" s="0" t="n">
-        <v>-1</v>
+        <v>1800</v>
       </c>
       <c r="G72" s="4" t="n"/>
       <c r="H72" s="4" t="n"/>
@@ -2258,25 +2266,409 @@
     </row>
     <row r="73">
       <c r="B73" s="0" t="n">
-        <v>9200</v>
+        <v>1820</v>
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>narrator</t>
+          <t>npc_jumpropekid</t>
         </is>
       </c>
       <c r="D73" s="4" t="n"/>
       <c r="E73" s="4" t="inlineStr">
         <is>
-          <t>@dialogue.9200</t>
+          <t>@dialogue.common.no_clue</t>
         </is>
       </c>
       <c r="F73" s="0" t="n">
-        <v>-1</v>
+        <v>1800</v>
       </c>
       <c r="G73" s="4" t="n"/>
       <c r="H73" s="4" t="n"/>
       <c r="I73" s="4" t="n"/>
+    </row>
+    <row r="74">
+      <c r="B74" t="n">
+        <v>1830</v>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>npc_jumpropekid</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="n"/>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.1830</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G74" s="4" t="n"/>
+      <c r="H74" s="4" t="n"/>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t>startQuest:102</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" t="n">
+        <v>9000</v>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="n"/>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9000</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>9001</v>
+      </c>
+      <c r="G75" s="4" t="n"/>
+      <c r="H75" s="4" t="n"/>
+      <c r="I75" s="4" t="n"/>
+    </row>
+    <row r="76">
+      <c r="B76" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="n"/>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9001</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>9002</v>
+      </c>
+      <c r="G76" s="4" t="n"/>
+      <c r="H76" s="4" t="n"/>
+      <c r="I76" s="4" t="n"/>
+    </row>
+    <row r="77">
+      <c r="B77" t="n">
+        <v>9002</v>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="n"/>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9002</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G77" s="4" t="n"/>
+      <c r="H77" s="4" t="n"/>
+      <c r="I77" s="4" t="n"/>
+    </row>
+    <row r="78">
+      <c r="B78" t="n">
+        <v>9010</v>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>npc_mayor</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>촌장</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9010</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>9011</v>
+      </c>
+      <c r="G78" s="4" t="n"/>
+      <c r="H78" s="4" t="n"/>
+      <c r="I78" s="4" t="n"/>
+    </row>
+    <row r="79">
+      <c r="B79" t="n">
+        <v>9011</v>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>npc_mayor</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>촌장</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9011</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>9012</v>
+      </c>
+      <c r="G79" s="4" t="n"/>
+      <c r="H79" s="4" t="n"/>
+      <c r="I79" s="4" t="n"/>
+    </row>
+    <row r="80">
+      <c r="B80" t="n">
+        <v>9012</v>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>npc_mayor</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>촌장</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9012</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>9013</v>
+      </c>
+      <c r="G80" s="4" t="n"/>
+      <c r="H80" s="4" t="n"/>
+      <c r="I80" s="4" t="n"/>
+    </row>
+    <row r="81">
+      <c r="B81" t="n">
+        <v>9013</v>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>npc_mayor</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>촌장</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9013</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G81" s="4" t="n"/>
+      <c r="H81" s="4" t="n"/>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>meet:npc_mayor;addNote:101;startQuest:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" t="n">
+        <v>9020</v>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="n"/>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9020</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>9021</v>
+      </c>
+      <c r="G82" s="4" t="n"/>
+      <c r="H82" s="4" t="n"/>
+      <c r="I82" s="4" t="n"/>
+    </row>
+    <row r="83">
+      <c r="B83" t="n">
+        <v>9021</v>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="n"/>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9021</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>9022</v>
+      </c>
+      <c r="G83" s="4" t="n"/>
+      <c r="H83" s="4" t="n"/>
+      <c r="I83" s="4" t="n"/>
+    </row>
+    <row r="84">
+      <c r="B84" t="n">
+        <v>9022</v>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="n"/>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9022</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G84" s="4" t="n"/>
+      <c r="H84" s="4" t="n"/>
+      <c r="I84" s="4" t="n"/>
+    </row>
+    <row r="85">
+      <c r="B85" t="n">
+        <v>9100</v>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="n"/>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9100</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>9101,9102</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="n"/>
+      <c r="I85" s="4" t="n"/>
+    </row>
+    <row r="86">
+      <c r="B86" t="n">
+        <v>9101</v>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="n"/>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9101</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>9103</v>
+      </c>
+      <c r="G86" s="4" t="n"/>
+      <c r="H86" s="4" t="n"/>
+      <c r="I86" s="4" t="inlineStr">
+        <is>
+          <t>save</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" t="n">
+        <v>9102</v>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="n"/>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9102</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G87" s="4" t="n"/>
+      <c r="H87" s="4" t="n"/>
+      <c r="I87" s="4" t="n"/>
+    </row>
+    <row r="88">
+      <c r="B88" t="n">
+        <v>9103</v>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="n"/>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9103</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G88" s="4" t="n"/>
+      <c r="H88" s="4" t="n"/>
+      <c r="I88" s="4" t="n"/>
+    </row>
+    <row r="89">
+      <c r="B89" t="n">
+        <v>9200</v>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="n"/>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>@dialogue.9200</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G89" s="4" t="n"/>
+      <c r="H89" s="4" t="n"/>
+      <c r="I89" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
refactor(table): text columns use Text keys only; generate RowData fields from schema
- Move literal text in Notebook, Quest, QuestObjective and Dialogue
  SpeakerName into Text tables (new Text_Notebook part) and reference by @key.
- Validator rejects literal text in textKey columns.
- convert_table.py generates Scripts/Data/Table/Generated/{rowClass}.cs
  (partial, fields from schema columns, schema "default" as initializer);
  hand-written row classes keep only constants and methods.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Table/Excel/Dialogue.xlsx
+++ b/Table/Excel/Dialogue.xlsx
@@ -2287,7 +2287,7 @@
       <c r="I73" s="4" t="n"/>
     </row>
     <row r="74">
-      <c r="B74" t="n">
+      <c r="B74" s="0" t="n">
         <v>1830</v>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -2301,7 +2301,7 @@
           <t>@dialogue.1830</t>
         </is>
       </c>
-      <c r="F74" t="n">
+      <c r="F74" s="0" t="n">
         <v>1800</v>
       </c>
       <c r="G74" s="4" t="n"/>
@@ -2313,7 +2313,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="B75" t="n">
+      <c r="B75" s="0" t="n">
         <v>9000</v>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -2327,7 +2327,7 @@
           <t>@dialogue.9000</t>
         </is>
       </c>
-      <c r="F75" t="n">
+      <c r="F75" s="0" t="n">
         <v>9001</v>
       </c>
       <c r="G75" s="4" t="n"/>
@@ -2335,7 +2335,7 @@
       <c r="I75" s="4" t="n"/>
     </row>
     <row r="76">
-      <c r="B76" t="n">
+      <c r="B76" s="0" t="n">
         <v>9001</v>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -2349,7 +2349,7 @@
           <t>@dialogue.9001</t>
         </is>
       </c>
-      <c r="F76" t="n">
+      <c r="F76" s="0" t="n">
         <v>9002</v>
       </c>
       <c r="G76" s="4" t="n"/>
@@ -2357,7 +2357,7 @@
       <c r="I76" s="4" t="n"/>
     </row>
     <row r="77">
-      <c r="B77" t="n">
+      <c r="B77" s="0" t="n">
         <v>9002</v>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -2371,7 +2371,7 @@
           <t>@dialogue.9002</t>
         </is>
       </c>
-      <c r="F77" t="n">
+      <c r="F77" s="0" t="n">
         <v>-1</v>
       </c>
       <c r="G77" s="4" t="n"/>
@@ -2379,7 +2379,7 @@
       <c r="I77" s="4" t="n"/>
     </row>
     <row r="78">
-      <c r="B78" t="n">
+      <c r="B78" s="0" t="n">
         <v>9010</v>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>촌장</t>
+          <t>@character.mayor.name</t>
         </is>
       </c>
       <c r="E78" s="4" t="inlineStr">
@@ -2397,7 +2397,7 @@
           <t>@dialogue.9010</t>
         </is>
       </c>
-      <c r="F78" t="n">
+      <c r="F78" s="0" t="n">
         <v>9011</v>
       </c>
       <c r="G78" s="4" t="n"/>
@@ -2405,7 +2405,7 @@
       <c r="I78" s="4" t="n"/>
     </row>
     <row r="79">
-      <c r="B79" t="n">
+      <c r="B79" s="0" t="n">
         <v>9011</v>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -2415,7 +2415,7 @@
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>촌장</t>
+          <t>@character.mayor.name</t>
         </is>
       </c>
       <c r="E79" s="4" t="inlineStr">
@@ -2423,7 +2423,7 @@
           <t>@dialogue.9011</t>
         </is>
       </c>
-      <c r="F79" t="n">
+      <c r="F79" s="0" t="n">
         <v>9012</v>
       </c>
       <c r="G79" s="4" t="n"/>
@@ -2431,7 +2431,7 @@
       <c r="I79" s="4" t="n"/>
     </row>
     <row r="80">
-      <c r="B80" t="n">
+      <c r="B80" s="0" t="n">
         <v>9012</v>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>촌장</t>
+          <t>@character.mayor.name</t>
         </is>
       </c>
       <c r="E80" s="4" t="inlineStr">
@@ -2449,7 +2449,7 @@
           <t>@dialogue.9012</t>
         </is>
       </c>
-      <c r="F80" t="n">
+      <c r="F80" s="0" t="n">
         <v>9013</v>
       </c>
       <c r="G80" s="4" t="n"/>
@@ -2457,7 +2457,7 @@
       <c r="I80" s="4" t="n"/>
     </row>
     <row r="81">
-      <c r="B81" t="n">
+      <c r="B81" s="0" t="n">
         <v>9013</v>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>촌장</t>
+          <t>@character.mayor.name</t>
         </is>
       </c>
       <c r="E81" s="4" t="inlineStr">
@@ -2475,7 +2475,7 @@
           <t>@dialogue.9013</t>
         </is>
       </c>
-      <c r="F81" t="n">
+      <c r="F81" s="0" t="n">
         <v>-1</v>
       </c>
       <c r="G81" s="4" t="n"/>
@@ -2487,7 +2487,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="B82" t="n">
+      <c r="B82" s="0" t="n">
         <v>9020</v>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -2501,7 +2501,7 @@
           <t>@dialogue.9020</t>
         </is>
       </c>
-      <c r="F82" t="n">
+      <c r="F82" s="0" t="n">
         <v>9021</v>
       </c>
       <c r="G82" s="4" t="n"/>
@@ -2509,7 +2509,7 @@
       <c r="I82" s="4" t="n"/>
     </row>
     <row r="83">
-      <c r="B83" t="n">
+      <c r="B83" s="0" t="n">
         <v>9021</v>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -2523,7 +2523,7 @@
           <t>@dialogue.9021</t>
         </is>
       </c>
-      <c r="F83" t="n">
+      <c r="F83" s="0" t="n">
         <v>9022</v>
       </c>
       <c r="G83" s="4" t="n"/>
@@ -2531,7 +2531,7 @@
       <c r="I83" s="4" t="n"/>
     </row>
     <row r="84">
-      <c r="B84" t="n">
+      <c r="B84" s="0" t="n">
         <v>9022</v>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -2545,7 +2545,7 @@
           <t>@dialogue.9022</t>
         </is>
       </c>
-      <c r="F84" t="n">
+      <c r="F84" s="0" t="n">
         <v>-1</v>
       </c>
       <c r="G84" s="4" t="n"/>
@@ -2553,7 +2553,7 @@
       <c r="I84" s="4" t="n"/>
     </row>
     <row r="85">
-      <c r="B85" t="n">
+      <c r="B85" s="0" t="n">
         <v>9100</v>
       </c>
       <c r="C85" s="4" t="inlineStr">
@@ -2567,7 +2567,7 @@
           <t>@dialogue.9100</t>
         </is>
       </c>
-      <c r="F85" t="n">
+      <c r="F85" s="0" t="n">
         <v>-1</v>
       </c>
       <c r="G85" s="4" t="inlineStr">
@@ -2579,7 +2579,7 @@
       <c r="I85" s="4" t="n"/>
     </row>
     <row r="86">
-      <c r="B86" t="n">
+      <c r="B86" s="0" t="n">
         <v>9101</v>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -2593,7 +2593,7 @@
           <t>@dialogue.9101</t>
         </is>
       </c>
-      <c r="F86" t="n">
+      <c r="F86" s="0" t="n">
         <v>9103</v>
       </c>
       <c r="G86" s="4" t="n"/>
@@ -2605,7 +2605,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="B87" t="n">
+      <c r="B87" s="0" t="n">
         <v>9102</v>
       </c>
       <c r="C87" s="4" t="inlineStr">
@@ -2619,7 +2619,7 @@
           <t>@dialogue.9102</t>
         </is>
       </c>
-      <c r="F87" t="n">
+      <c r="F87" s="0" t="n">
         <v>-1</v>
       </c>
       <c r="G87" s="4" t="n"/>
@@ -2627,7 +2627,7 @@
       <c r="I87" s="4" t="n"/>
     </row>
     <row r="88">
-      <c r="B88" t="n">
+      <c r="B88" s="0" t="n">
         <v>9103</v>
       </c>
       <c r="C88" s="4" t="inlineStr">
@@ -2641,7 +2641,7 @@
           <t>@dialogue.9103</t>
         </is>
       </c>
-      <c r="F88" t="n">
+      <c r="F88" s="0" t="n">
         <v>-1</v>
       </c>
       <c r="G88" s="4" t="n"/>
@@ -2649,7 +2649,7 @@
       <c r="I88" s="4" t="n"/>
     </row>
     <row r="89">
-      <c r="B89" t="n">
+      <c r="B89" s="0" t="n">
         <v>9200</v>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -2663,7 +2663,7 @@
           <t>@dialogue.9200</t>
         </is>
       </c>
-      <c r="F89" t="n">
+      <c r="F89" s="0" t="n">
         <v>-1</v>
       </c>
       <c r="G89" s="4" t="n"/>

</xml_diff>